<commit_message>
segunda version casi lista xd
</commit_message>
<xml_diff>
--- a/temp_mhr/desasignar_53072529.xlsx
+++ b/temp_mhr/desasignar_53072529.xlsx
@@ -470,7 +470,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>700161071</t>
+          <t>700179112</t>
         </is>
       </c>
     </row>
@@ -487,7 +487,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>501140686</t>
+          <t>501157977</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>700160254</t>
+          <t>700172268</t>
         </is>
       </c>
     </row>
@@ -521,7 +521,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>501139829</t>
+          <t>501151373</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>700175726</t>
+          <t>700177918</t>
         </is>
       </c>
     </row>
@@ -589,7 +589,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>501154901</t>
+          <t>501156823</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>700180042</t>
+          <t>700167289</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>501158917</t>
+          <t>501146304</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>700177311</t>
+          <t>700170982</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>501156216</t>
+          <t>501150067</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>700177680</t>
+          <t>700179264</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>501156585</t>
+          <t>501158129</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>700178492</t>
+          <t>700177681</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>501157357</t>
+          <t>501156586</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>700158121</t>
+          <t>700167288</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>501137986</t>
+          <t>501146303</t>
         </is>
       </c>
     </row>
@@ -776,7 +776,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>700177004</t>
+          <t>700175777</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>501155899</t>
+          <t>501154952</t>
         </is>
       </c>
     </row>
@@ -810,7 +810,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>700178130</t>
+          <t>700162037</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>501156995</t>
+          <t>501141712</t>
         </is>
       </c>
     </row>
@@ -844,7 +844,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>700158115</t>
+          <t>700161072</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>501137980</t>
+          <t>501140687</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>700179117</t>
+          <t>700161461</t>
         </is>
       </c>
     </row>
@@ -895,7 +895,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>501157982</t>
+          <t>501141076</t>
         </is>
       </c>
     </row>
@@ -912,7 +912,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>700180033</t>
+          <t>700179573</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>501158908</t>
+          <t>501158448</t>
         </is>
       </c>
     </row>
@@ -946,7 +946,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>700162521</t>
+          <t>700161536</t>
         </is>
       </c>
     </row>
@@ -963,7 +963,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>501142226</t>
+          <t>501141171</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>700170982</t>
+          <t>700180031</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>501150067</t>
+          <t>501158906</t>
         </is>
       </c>
     </row>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>700174724</t>
+          <t>700169346</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>501153879</t>
+          <t>501148401</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>700165633</t>
+          <t>700174383</t>
         </is>
       </c>
     </row>
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>501144628</t>
+          <t>501153528</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>700178131</t>
+          <t>700174384</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>501156996</t>
+          <t>501153529</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>700162036</t>
+          <t>700177638</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>501141711</t>
+          <t>501156543</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>700177642</t>
+          <t>700175726</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>501156547</t>
+          <t>501154901</t>
         </is>
       </c>
     </row>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>700176148</t>
+          <t>700167283</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>501155323</t>
+          <t>501146298</t>
         </is>
       </c>
     </row>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>700177903</t>
+          <t>700179708</t>
         </is>
       </c>
     </row>
@@ -1235,7 +1235,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>501156808</t>
+          <t>501158583</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>700180031</t>
+          <t>700158789</t>
         </is>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>501158906</t>
+          <t>501138633</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>700178790</t>
+          <t>700174493</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>501157665</t>
+          <t>501153638</t>
         </is>
       </c>
     </row>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>700169345</t>
+          <t>700177642</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>501148400</t>
+          <t>501156547</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>700173532</t>
+          <t>700177270</t>
         </is>
       </c>
     </row>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>501152667</t>
+          <t>501156175</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>700177331</t>
+          <t>700176289</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>501156236</t>
+          <t>501155484</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1422,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>700179115</t>
+          <t>700175776</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>501157980</t>
+          <t>501154951</t>
         </is>
       </c>
     </row>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>700176043</t>
+          <t>700177307</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>501155218</t>
+          <t>501156212</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>700177902</t>
+          <t>700178788</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>501156807</t>
+          <t>501157663</t>
         </is>
       </c>
     </row>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>700178223</t>
+          <t>700173255</t>
         </is>
       </c>
     </row>
@@ -1541,7 +1541,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>501157088</t>
+          <t>501152380</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>700174712</t>
+          <t>700179620</t>
         </is>
       </c>
     </row>
@@ -1575,7 +1575,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>501153857</t>
+          <t>501158495</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>700162386</t>
+          <t>700156870</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>501142091</t>
+          <t>501136725</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>700158789</t>
+          <t>700178789</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>501138633</t>
+          <t>501157664</t>
         </is>
       </c>
     </row>
@@ -1660,7 +1660,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>700175725</t>
+          <t>700172038</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1677,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>501154900</t>
+          <t>501151143</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1694,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>700180073</t>
+          <t>700177108</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>501158938</t>
+          <t>501156013</t>
         </is>
       </c>
     </row>
@@ -1728,7 +1728,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>700177895</t>
+          <t>700177105</t>
         </is>
       </c>
     </row>
@@ -1745,7 +1745,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>501156800</t>
+          <t>501156010</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>700177304</t>
+          <t>700160254</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1779,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>501156209</t>
+          <t>501139829</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1796,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>700162041</t>
+          <t>700173850</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>501141716</t>
+          <t>501152975</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>700179218</t>
+          <t>700167282</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>501158083</t>
+          <t>501146297</t>
         </is>
       </c>
     </row>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>700166265</t>
+          <t>700177309</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>501145260</t>
+          <t>501156214</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>700175777</t>
+          <t>700178503</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>501154952</t>
+          <t>501157368</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>700178275</t>
+          <t>700177308</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>501157140</t>
+          <t>501156213</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>700177987</t>
+          <t>700167137</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>501156842</t>
+          <t>501146142</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>700169346</t>
+          <t>700178578</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>501148401</t>
+          <t>501157443</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>700159761</t>
+          <t>700177004</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>501139673</t>
+          <t>501155899</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>700177069</t>
+          <t>700177727</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2085,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>501155967</t>
+          <t>501156632</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>700174593</t>
+          <t>700177070</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2119,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>501153748</t>
+          <t>501155988</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2136,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>700177309</t>
+          <t>700172574</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>501156214</t>
+          <t>501151689</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>700167137</t>
+          <t>700177303</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>501146142</t>
+          <t>501156208</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>700177307</t>
+          <t>700176946</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>501156212</t>
+          <t>501155841</t>
         </is>
       </c>
     </row>
@@ -2238,7 +2238,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>700175758</t>
+          <t>700162036</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>501154933</t>
+          <t>501141711</t>
         </is>
       </c>
     </row>
@@ -2272,7 +2272,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>700176946</t>
+          <t>700168420</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>501155841</t>
+          <t>501147465</t>
         </is>
       </c>
     </row>
@@ -2306,7 +2306,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>700179533</t>
+          <t>700174593</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>501158408</t>
+          <t>501153748</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>700178505</t>
+          <t>700178806</t>
         </is>
       </c>
     </row>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>501157370</t>
+          <t>501157671</t>
         </is>
       </c>
     </row>
@@ -2374,7 +2374,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>700177731</t>
+          <t>700158786</t>
         </is>
       </c>
     </row>
@@ -2391,7 +2391,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>501156636</t>
+          <t>501138630</t>
         </is>
       </c>
     </row>
@@ -2408,7 +2408,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>700158786</t>
+          <t>700179545</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2425,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>501138630</t>
+          <t>501158420</t>
         </is>
       </c>
     </row>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>700161461</t>
+          <t>700178579</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>501141076</t>
+          <t>501157444</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2476,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>700174384</t>
+          <t>700177728</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>501153529</t>
+          <t>501156633</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>700176289</t>
+          <t>700173532</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>501155484</t>
+          <t>501152667</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>700180030</t>
+          <t>700178275</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>501158905</t>
+          <t>501157140</t>
         </is>
       </c>
     </row>
@@ -2578,7 +2578,7 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>700173255</t>
+          <t>700174723</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="C127" s="2" t="inlineStr">
         <is>
-          <t>501152380</t>
+          <t>501153878</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>700177638</t>
+          <t>700172036</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2629,7 @@
       </c>
       <c r="C129" s="2" t="inlineStr">
         <is>
-          <t>501156543</t>
+          <t>501151141</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>700157674</t>
+          <t>700174411</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>501137509</t>
+          <t>501153556</t>
         </is>
       </c>
     </row>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>700170514</t>
+          <t>700177673</t>
         </is>
       </c>
     </row>
@@ -2731,7 +2731,7 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>501149589</t>
+          <t>501156578</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>700175759</t>
+          <t>700173796</t>
         </is>
       </c>
     </row>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>501154934</t>
+          <t>501152921</t>
         </is>
       </c>
     </row>
@@ -2782,7 +2782,7 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>700177681</t>
+          <t>700177684</t>
         </is>
       </c>
     </row>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="C139" s="2" t="inlineStr">
         <is>
-          <t>501156586</t>
+          <t>501156589</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
       </c>
       <c r="C140" s="2" t="inlineStr">
         <is>
-          <t>700172035</t>
+          <t>700162520</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2833,7 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>501151140</t>
+          <t>501142225</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="C142" s="2" t="inlineStr">
         <is>
-          <t>700177322</t>
+          <t>700180041</t>
         </is>
       </c>
     </row>
@@ -2867,7 +2867,7 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>501156227</t>
+          <t>501158916</t>
         </is>
       </c>
     </row>
@@ -2884,7 +2884,7 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>700177464</t>
+          <t>700158787</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2901,7 @@
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>501156369</t>
+          <t>501138631</t>
         </is>
       </c>
     </row>
@@ -2918,7 +2918,7 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>700178806</t>
+          <t>700177916</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>501157671</t>
+          <t>501156821</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>700166080</t>
+          <t>700177464</t>
         </is>
       </c>
     </row>
@@ -2969,7 +2969,7 @@
       </c>
       <c r="C149" s="2" t="inlineStr">
         <is>
-          <t>501145085</t>
+          <t>501156369</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="C150" s="2" t="inlineStr">
         <is>
-          <t>700177918</t>
+          <t>700176047</t>
         </is>
       </c>
     </row>
@@ -3003,7 +3003,7 @@
       </c>
       <c r="C151" s="2" t="inlineStr">
         <is>
-          <t>501156823</t>
+          <t>501155222</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="C152" s="2" t="inlineStr">
         <is>
-          <t>700179574</t>
+          <t>700165716</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>501158449</t>
+          <t>501144721</t>
         </is>
       </c>
     </row>
@@ -3054,7 +3054,7 @@
       </c>
       <c r="C154" s="2" t="inlineStr">
         <is>
-          <t>700176947</t>
+          <t>700156837</t>
         </is>
       </c>
     </row>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>501155842</t>
+          <t>501136682</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>700177721</t>
+          <t>700161537</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3105,7 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>501156626</t>
+          <t>501141172</t>
         </is>
       </c>
     </row>
@@ -3122,7 +3122,7 @@
       </c>
       <c r="C158" s="2" t="inlineStr">
         <is>
-          <t>700174723</t>
+          <t>700177304</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3139,7 @@
       </c>
       <c r="C159" s="2" t="inlineStr">
         <is>
-          <t>501153878</t>
+          <t>501156209</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="C160" s="2" t="inlineStr">
         <is>
-          <t>700178230</t>
+          <t>700160255</t>
         </is>
       </c>
     </row>
@@ -3173,7 +3173,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>501157095</t>
+          <t>501139830</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="C162" s="2" t="inlineStr">
         <is>
-          <t>700179708</t>
+          <t>700156836</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>501158583</t>
+          <t>501136681</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>700170082</t>
+          <t>700157662</t>
         </is>
       </c>
     </row>
@@ -3241,7 +3241,7 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>501149147</t>
+          <t>501137497</t>
         </is>
       </c>
     </row>
@@ -3258,7 +3258,7 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>700176118</t>
+          <t>700170993</t>
         </is>
       </c>
     </row>
@@ -3275,7 +3275,7 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>501155293</t>
+          <t>501150078</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>700165716</t>
+          <t>700178688</t>
         </is>
       </c>
     </row>
@@ -3309,7 +3309,7 @@
       </c>
       <c r="C169" s="2" t="inlineStr">
         <is>
-          <t>501144721</t>
+          <t>501157563</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="C170" s="2" t="inlineStr">
         <is>
-          <t>700167283</t>
+          <t>700178790</t>
         </is>
       </c>
     </row>
@@ -3343,7 +3343,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>501146298</t>
+          <t>501157665</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>700165628</t>
+          <t>700177331</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>501144623</t>
+          <t>501156236</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>700178788</t>
+          <t>700179218</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>501157663</t>
+          <t>501158083</t>
         </is>
       </c>
     </row>
@@ -3428,7 +3428,7 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>700175794</t>
+          <t>700157673</t>
         </is>
       </c>
     </row>
@@ -3445,7 +3445,7 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>501154959</t>
+          <t>501137508</t>
         </is>
       </c>
     </row>
@@ -3462,7 +3462,7 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>700162040</t>
+          <t>700177986</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>501141715</t>
+          <t>501156841</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3496,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>700173939</t>
+          <t>700178274</t>
         </is>
       </c>
     </row>
@@ -3513,7 +3513,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>501153074</t>
+          <t>501157139</t>
         </is>
       </c>
     </row>
@@ -3530,7 +3530,7 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>700177003</t>
+          <t>700177722</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>501155898</t>
+          <t>501156627</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>700177916</t>
+          <t>700176012</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>501156821</t>
+          <t>501155187</t>
         </is>
       </c>
     </row>
@@ -3598,7 +3598,7 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>700161073</t>
+          <t>700178687</t>
         </is>
       </c>
     </row>
@@ -3615,7 +3615,7 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>501140688</t>
+          <t>501157562</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3632,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>700163414</t>
+          <t>700177987</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3649,7 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>501143369</t>
+          <t>501156842</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3666,7 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>700177005</t>
+          <t>700180030</t>
         </is>
       </c>
     </row>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>501155900</t>
+          <t>501158905</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3700,7 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>700178503</t>
+          <t>700176044</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>501157368</t>
+          <t>501155219</t>
         </is>
       </c>
     </row>
@@ -3734,7 +3734,7 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>700178787</t>
+          <t>700173797</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>501157662</t>
+          <t>501152922</t>
         </is>
       </c>
     </row>
@@ -3768,7 +3768,7 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>700162385</t>
+          <t>700167136</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3785,7 @@
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>501142090</t>
+          <t>501146141</t>
         </is>
       </c>
     </row>
@@ -3802,7 +3802,7 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>700162038</t>
+          <t>700173939</t>
         </is>
       </c>
     </row>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>501141713</t>
+          <t>501153074</t>
         </is>
       </c>
     </row>
@@ -3836,7 +3836,7 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>700166266</t>
+          <t>700177729</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>501145261</t>
+          <t>501156634</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3870,7 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>700162037</t>
+          <t>700162038</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>501141712</t>
+          <t>501141713</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3904,7 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>700179116</t>
+          <t>700175778</t>
         </is>
       </c>
     </row>
@@ -3921,7 +3921,7 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>501157981</t>
+          <t>501154953</t>
         </is>
       </c>
     </row>
@@ -3938,7 +3938,7 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>700179620</t>
+          <t>700178787</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3955,7 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>501158495</t>
+          <t>501157662</t>
         </is>
       </c>
     </row>
@@ -3972,7 +3972,7 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>700167136</t>
+          <t>700077051</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>501146141</t>
+          <t>501035585</t>
         </is>
       </c>
     </row>
@@ -4006,7 +4006,7 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>700177673</t>
+          <t>700176145</t>
         </is>
       </c>
     </row>
@@ -4023,7 +4023,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>501156578</t>
+          <t>501155320</t>
         </is>
       </c>
     </row>
@@ -4040,7 +4040,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>700177728</t>
+          <t>700177721</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>501156633</t>
+          <t>501156626</t>
         </is>
       </c>
     </row>
@@ -4074,7 +4074,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>700161494</t>
+          <t>700175758</t>
         </is>
       </c>
     </row>
@@ -4091,7 +4091,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>501141109</t>
+          <t>501154933</t>
         </is>
       </c>
     </row>
@@ -4108,7 +4108,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>700178578</t>
+          <t>700170514</t>
         </is>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>501157443</t>
+          <t>501149589</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>700174494</t>
+          <t>700175760</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4159,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>501153639</t>
+          <t>501154935</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>700176044</t>
+          <t>700178599</t>
         </is>
       </c>
     </row>
@@ -4193,7 +4193,7 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>501155219</t>
+          <t>501157466</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="C222" s="2" t="inlineStr">
         <is>
-          <t>700156749</t>
+          <t>700168419</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4227,7 @@
       </c>
       <c r="C223" s="2" t="inlineStr">
         <is>
-          <t>501136584</t>
+          <t>501147464</t>
         </is>
       </c>
     </row>
@@ -4244,7 +4244,7 @@
       </c>
       <c r="C224" s="2" t="inlineStr">
         <is>
-          <t>700160255</t>
+          <t>700176933</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="C225" s="2" t="inlineStr">
         <is>
-          <t>501139830</t>
+          <t>501155828</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="C226" s="2" t="inlineStr">
         <is>
-          <t>700178688</t>
+          <t>700172267</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4295,7 @@
       </c>
       <c r="C227" s="2" t="inlineStr">
         <is>
-          <t>501157563</t>
+          <t>501151372</t>
         </is>
       </c>
     </row>
@@ -4312,7 +4312,7 @@
       </c>
       <c r="C228" s="2" t="inlineStr">
         <is>
-          <t>700156869</t>
+          <t>700159804</t>
         </is>
       </c>
     </row>
@@ -4329,7 +4329,7 @@
       </c>
       <c r="C229" s="2" t="inlineStr">
         <is>
-          <t>501136724</t>
+          <t>501139679</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="C230" s="2" t="inlineStr">
         <is>
-          <t>700177108</t>
+          <t>700175793</t>
         </is>
       </c>
     </row>
@@ -4363,7 +4363,7 @@
       </c>
       <c r="C231" s="2" t="inlineStr">
         <is>
-          <t>501156013</t>
+          <t>501154958</t>
         </is>
       </c>
     </row>
@@ -4380,7 +4380,7 @@
       </c>
       <c r="C232" s="2" t="inlineStr">
         <is>
-          <t>700177306</t>
+          <t>700180032</t>
         </is>
       </c>
     </row>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="C233" s="2" t="inlineStr">
         <is>
-          <t>501156211</t>
+          <t>501158907</t>
         </is>
       </c>
     </row>
@@ -4414,7 +4414,7 @@
       </c>
       <c r="C234" s="2" t="inlineStr">
         <is>
-          <t>700175779</t>
+          <t>700175759</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="C235" s="2" t="inlineStr">
         <is>
-          <t>501154954</t>
+          <t>501154934</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="C236" s="2" t="inlineStr">
         <is>
-          <t>700077051</t>
+          <t>700170082</t>
         </is>
       </c>
     </row>
@@ -4465,7 +4465,7 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>501035585</t>
+          <t>501149147</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>700177107</t>
+          <t>700179117</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>501156012</t>
+          <t>501157982</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4516,7 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>700175760</t>
+          <t>700178504</t>
         </is>
       </c>
     </row>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>501154935</t>
+          <t>501157369</t>
         </is>
       </c>
     </row>
@@ -4550,7 +4550,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>700175761</t>
+          <t>700162521</t>
         </is>
       </c>
     </row>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>501154936</t>
+          <t>501142226</t>
         </is>
       </c>
     </row>
@@ -4584,7 +4584,7 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>700177726</t>
+          <t>700176290</t>
         </is>
       </c>
     </row>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>501156631</t>
+          <t>501155485</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4618,7 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>700177109</t>
+          <t>700173849</t>
         </is>
       </c>
     </row>
@@ -4635,7 +4635,7 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>501156014</t>
+          <t>501152974</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4652,7 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>700167288</t>
+          <t>700156869</t>
         </is>
       </c>
     </row>
@@ -4669,7 +4669,7 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>501146303</t>
+          <t>501136724</t>
         </is>
       </c>
     </row>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>700177639</t>
+          <t>700177915</t>
         </is>
       </c>
     </row>
@@ -4703,7 +4703,7 @@
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>501156544</t>
+          <t>501156820</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       </c>
       <c r="C252" s="2" t="inlineStr">
         <is>
-          <t>700163413</t>
+          <t>700180074</t>
         </is>
       </c>
     </row>
@@ -4737,7 +4737,7 @@
       </c>
       <c r="C253" s="2" t="inlineStr">
         <is>
-          <t>501143368</t>
+          <t>501158939</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4754,7 @@
       </c>
       <c r="C254" s="2" t="inlineStr">
         <is>
-          <t>700157661</t>
+          <t>700172037</t>
         </is>
       </c>
     </row>
@@ -4771,7 +4771,7 @@
       </c>
       <c r="C255" s="2" t="inlineStr">
         <is>
-          <t>501137496</t>
+          <t>501151142</t>
         </is>
       </c>
     </row>
@@ -4788,7 +4788,7 @@
       </c>
       <c r="C256" s="2" t="inlineStr">
         <is>
-          <t>700170993</t>
+          <t>700179115</t>
         </is>
       </c>
     </row>
@@ -4805,7 +4805,7 @@
       </c>
       <c r="C257" s="2" t="inlineStr">
         <is>
-          <t>501150078</t>
+          <t>501157980</t>
         </is>
       </c>
     </row>
@@ -4822,7 +4822,7 @@
       </c>
       <c r="C258" s="2" t="inlineStr">
         <is>
-          <t>700177722</t>
+          <t>700163189</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="C259" s="2" t="inlineStr">
         <is>
-          <t>501156627</t>
+          <t>501143134</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="C260" s="2" t="inlineStr">
         <is>
-          <t>700177110</t>
+          <t>700179113</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4873,7 @@
       </c>
       <c r="C261" s="2" t="inlineStr">
         <is>
-          <t>501156015</t>
+          <t>501157978</t>
         </is>
       </c>
     </row>
@@ -4890,7 +4890,7 @@
       </c>
       <c r="C262" s="2" t="inlineStr">
         <is>
-          <t>700179264</t>
+          <t>700177677</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
       </c>
       <c r="C263" s="2" t="inlineStr">
         <is>
-          <t>501158129</t>
+          <t>501156583</t>
         </is>
       </c>
     </row>
@@ -4924,7 +4924,7 @@
       </c>
       <c r="C264" s="2" t="inlineStr">
         <is>
-          <t>700162520</t>
+          <t>700180528</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4941,7 @@
       </c>
       <c r="C265" s="2" t="inlineStr">
         <is>
-          <t>501142225</t>
+          <t>501159413</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C266" s="2" t="inlineStr">
         <is>
-          <t>700172268</t>
+          <t>700163413</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4975,7 @@
       </c>
       <c r="C267" s="2" t="inlineStr">
         <is>
-          <t>501151373</t>
+          <t>501143368</t>
         </is>
       </c>
     </row>
@@ -4992,7 +4992,7 @@
       </c>
       <c r="C268" s="2" t="inlineStr">
         <is>
-          <t>700176147</t>
+          <t>700177110</t>
         </is>
       </c>
     </row>
@@ -5009,7 +5009,7 @@
       </c>
       <c r="C269" s="2" t="inlineStr">
         <is>
-          <t>501155322</t>
+          <t>501156015</t>
         </is>
       </c>
     </row>
@@ -5026,7 +5026,7 @@
       </c>
       <c r="C270" s="2" t="inlineStr">
         <is>
-          <t>700177308</t>
+          <t>700174494</t>
         </is>
       </c>
     </row>
@@ -5043,7 +5043,7 @@
       </c>
       <c r="C271" s="2" t="inlineStr">
         <is>
-          <t>501156213</t>
+          <t>501153639</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="C272" s="2" t="inlineStr">
         <is>
-          <t>700169347</t>
+          <t>700180530</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5077,7 @@
       </c>
       <c r="C273" s="2" t="inlineStr">
         <is>
-          <t>501148402</t>
+          <t>501159415</t>
         </is>
       </c>
     </row>
@@ -5094,7 +5094,7 @@
       </c>
       <c r="C274" s="2" t="inlineStr">
         <is>
-          <t>700174383</t>
+          <t>700172035</t>
         </is>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       </c>
       <c r="C275" s="2" t="inlineStr">
         <is>
-          <t>501153528</t>
+          <t>501151140</t>
         </is>
       </c>
     </row>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="C276" s="2" t="inlineStr">
         <is>
-          <t>700161493</t>
+          <t>700158121</t>
         </is>
       </c>
     </row>
@@ -5145,7 +5145,7 @@
       </c>
       <c r="C277" s="2" t="inlineStr">
         <is>
-          <t>501141108</t>
+          <t>501137986</t>
         </is>
       </c>
     </row>
@@ -5162,7 +5162,7 @@
       </c>
       <c r="C278" s="2" t="inlineStr">
         <is>
-          <t>700157608</t>
+          <t>700177003</t>
         </is>
       </c>
     </row>
@@ -5179,7 +5179,7 @@
       </c>
       <c r="C279" s="2" t="inlineStr">
         <is>
-          <t>501137443</t>
+          <t>501155898</t>
         </is>
       </c>
     </row>
@@ -5196,7 +5196,7 @@
       </c>
       <c r="C280" s="2" t="inlineStr">
         <is>
-          <t>700179268</t>
+          <t>700177109</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="C281" s="2" t="inlineStr">
         <is>
-          <t>501158133</t>
+          <t>501156014</t>
         </is>
       </c>
     </row>
@@ -5230,7 +5230,7 @@
       </c>
       <c r="C282" s="2" t="inlineStr">
         <is>
-          <t>700163189</t>
+          <t>700177322</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5247,7 @@
       </c>
       <c r="C283" s="2" t="inlineStr">
         <is>
-          <t>501143134</t>
+          <t>501156227</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="C284" s="2" t="inlineStr">
         <is>
-          <t>700159805</t>
+          <t>700176043</t>
         </is>
       </c>
     </row>
@@ -5281,7 +5281,7 @@
       </c>
       <c r="C285" s="2" t="inlineStr">
         <is>
-          <t>501139680</t>
+          <t>501155218</t>
         </is>
       </c>
     </row>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="C286" s="2" t="inlineStr">
         <is>
-          <t>700178229</t>
+          <t>700170081</t>
         </is>
       </c>
     </row>
@@ -5315,7 +5315,7 @@
       </c>
       <c r="C287" s="2" t="inlineStr">
         <is>
-          <t>501157094</t>
+          <t>501149146</t>
         </is>
       </c>
     </row>
@@ -5332,7 +5332,7 @@
       </c>
       <c r="C288" s="2" t="inlineStr">
         <is>
-          <t>700172036</t>
+          <t>700176147</t>
         </is>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
       </c>
       <c r="C289" s="2" t="inlineStr">
         <is>
-          <t>501151141</t>
+          <t>501155322</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5366,7 @@
       </c>
       <c r="C290" s="2" t="inlineStr">
         <is>
-          <t>700156870</t>
+          <t>700162040</t>
         </is>
       </c>
     </row>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C291" s="2" t="inlineStr">
         <is>
-          <t>501136725</t>
+          <t>501141715</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
       </c>
       <c r="C292" s="2" t="inlineStr">
         <is>
-          <t>700179114</t>
+          <t>700177002</t>
         </is>
       </c>
     </row>
@@ -5417,7 +5417,7 @@
       </c>
       <c r="C293" s="2" t="inlineStr">
         <is>
-          <t>501157979</t>
+          <t>501155897</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
       </c>
       <c r="C294" s="2" t="inlineStr">
         <is>
-          <t>700173849</t>
+          <t>700175779</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="C295" s="2" t="inlineStr">
         <is>
-          <t>501152974</t>
+          <t>501154954</t>
         </is>
       </c>
     </row>
@@ -5468,7 +5468,7 @@
       </c>
       <c r="C296" s="2" t="inlineStr">
         <is>
-          <t>700161536</t>
+          <t>700178229</t>
         </is>
       </c>
     </row>
@@ -5485,7 +5485,7 @@
       </c>
       <c r="C297" s="2" t="inlineStr">
         <is>
-          <t>501141171</t>
+          <t>501157094</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5502,7 @@
       </c>
       <c r="C298" s="2" t="inlineStr">
         <is>
-          <t>700157662</t>
+          <t>700180529</t>
         </is>
       </c>
     </row>
@@ -5519,7 +5519,7 @@
       </c>
       <c r="C299" s="2" t="inlineStr">
         <is>
-          <t>501137497</t>
+          <t>501159414</t>
         </is>
       </c>
     </row>
@@ -5536,7 +5536,7 @@
       </c>
       <c r="C300" s="2" t="inlineStr">
         <is>
-          <t>700176046</t>
+          <t>700174724</t>
         </is>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
       </c>
       <c r="C301" s="2" t="inlineStr">
         <is>
-          <t>501155221</t>
+          <t>501153879</t>
         </is>
       </c>
     </row>
@@ -5570,7 +5570,7 @@
       </c>
       <c r="C302" s="2" t="inlineStr">
         <is>
-          <t>700177729</t>
+          <t>700160396</t>
         </is>
       </c>
     </row>
@@ -5587,7 +5587,7 @@
       </c>
       <c r="C303" s="2" t="inlineStr">
         <is>
-          <t>501156634</t>
+          <t>501139971</t>
         </is>
       </c>
     </row>
@@ -5604,7 +5604,7 @@
       </c>
       <c r="C304" s="2" t="inlineStr">
         <is>
-          <t>700177271</t>
+          <t>700173940</t>
         </is>
       </c>
     </row>
@@ -5621,7 +5621,7 @@
       </c>
       <c r="C305" s="2" t="inlineStr">
         <is>
-          <t>501156176</t>
+          <t>501153075</t>
         </is>
       </c>
     </row>
@@ -5638,7 +5638,7 @@
       </c>
       <c r="C306" s="2" t="inlineStr">
         <is>
-          <t>700157660</t>
+          <t>700178223</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="C307" s="2" t="inlineStr">
         <is>
-          <t>501137495</t>
+          <t>501157088</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5672,7 @@
       </c>
       <c r="C308" s="2" t="inlineStr">
         <is>
-          <t>700174725</t>
+          <t>700179268</t>
         </is>
       </c>
     </row>
@@ -5689,7 +5689,7 @@
       </c>
       <c r="C309" s="2" t="inlineStr">
         <is>
-          <t>501153880</t>
+          <t>501158133</t>
         </is>
       </c>
     </row>
@@ -5706,7 +5706,7 @@
       </c>
       <c r="C310" s="2" t="inlineStr">
         <is>
-          <t>700178579</t>
+          <t>700158791</t>
         </is>
       </c>
     </row>
@@ -5723,7 +5723,7 @@
       </c>
       <c r="C311" s="2" t="inlineStr">
         <is>
-          <t>501157444</t>
+          <t>501138635</t>
         </is>
       </c>
     </row>
@@ -5740,7 +5740,7 @@
       </c>
       <c r="C312" s="2" t="inlineStr">
         <is>
-          <t>700177105</t>
+          <t>700157660</t>
         </is>
       </c>
     </row>
@@ -5757,7 +5757,7 @@
       </c>
       <c r="C313" s="2" t="inlineStr">
         <is>
-          <t>501156010</t>
+          <t>501137495</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="C314" s="2" t="inlineStr">
         <is>
-          <t>700178687</t>
+          <t>700174572</t>
         </is>
       </c>
     </row>
@@ -5791,7 +5791,7 @@
       </c>
       <c r="C315" s="2" t="inlineStr">
         <is>
-          <t>501157562</t>
+          <t>501153727</t>
         </is>
       </c>
     </row>
@@ -5808,7 +5808,7 @@
       </c>
       <c r="C316" s="2" t="inlineStr">
         <is>
-          <t>700175793</t>
+          <t>700172270</t>
         </is>
       </c>
     </row>
@@ -5825,7 +5825,7 @@
       </c>
       <c r="C317" s="2" t="inlineStr">
         <is>
-          <t>501154958</t>
+          <t>501151375</t>
         </is>
       </c>
     </row>
@@ -5842,7 +5842,7 @@
       </c>
       <c r="C318" s="2" t="inlineStr">
         <is>
-          <t>700178599</t>
+          <t>700177321</t>
         </is>
       </c>
     </row>
@@ -5859,7 +5859,7 @@
       </c>
       <c r="C319" s="2" t="inlineStr">
         <is>
-          <t>501157466</t>
+          <t>501156226</t>
         </is>
       </c>
     </row>
@@ -5876,7 +5876,7 @@
       </c>
       <c r="C320" s="2" t="inlineStr">
         <is>
-          <t>700172037</t>
+          <t>700177731</t>
         </is>
       </c>
     </row>
@@ -5893,7 +5893,7 @@
       </c>
       <c r="C321" s="2" t="inlineStr">
         <is>
-          <t>501151142</t>
+          <t>501156636</t>
         </is>
       </c>
     </row>
@@ -5910,7 +5910,7 @@
       </c>
       <c r="C322" s="2" t="inlineStr">
         <is>
-          <t>700178600</t>
+          <t>700174725</t>
         </is>
       </c>
     </row>
@@ -5927,7 +5927,7 @@
       </c>
       <c r="C323" s="2" t="inlineStr">
         <is>
-          <t>501157467</t>
+          <t>501153880</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5944,7 @@
       </c>
       <c r="C324" s="2" t="inlineStr">
         <is>
-          <t>700165715</t>
+          <t>700165633</t>
         </is>
       </c>
     </row>
@@ -5961,7 +5961,7 @@
       </c>
       <c r="C325" s="2" t="inlineStr">
         <is>
-          <t>501144720</t>
+          <t>501144628</t>
         </is>
       </c>
     </row>
@@ -5978,7 +5978,7 @@
       </c>
       <c r="C326" s="2" t="inlineStr">
         <is>
-          <t>700161537</t>
+          <t>700159761</t>
         </is>
       </c>
     </row>
@@ -5995,7 +5995,7 @@
       </c>
       <c r="C327" s="2" t="inlineStr">
         <is>
-          <t>501141172</t>
+          <t>501139673</t>
         </is>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       </c>
       <c r="C328" s="2" t="inlineStr">
         <is>
-          <t>700177684</t>
+          <t>700157661</t>
         </is>
       </c>
     </row>
@@ -6029,7 +6029,7 @@
       </c>
       <c r="C329" s="2" t="inlineStr">
         <is>
-          <t>501156589</t>
+          <t>501137496</t>
         </is>
       </c>
     </row>
@@ -6046,7 +6046,7 @@
       </c>
       <c r="C330" s="2" t="inlineStr">
         <is>
-          <t>700176011</t>
+          <t>700166265</t>
         </is>
       </c>
     </row>
@@ -6063,7 +6063,7 @@
       </c>
       <c r="C331" s="2" t="inlineStr">
         <is>
-          <t>501155186</t>
+          <t>501145260</t>
         </is>
       </c>
     </row>
@@ -6080,7 +6080,7 @@
       </c>
       <c r="C332" s="2" t="inlineStr">
         <is>
-          <t>700175781</t>
+          <t>700176011</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6097,7 @@
       </c>
       <c r="C333" s="2" t="inlineStr">
         <is>
-          <t>501154956</t>
+          <t>501155186</t>
         </is>
       </c>
     </row>
@@ -6114,7 +6114,7 @@
       </c>
       <c r="C334" s="2" t="inlineStr">
         <is>
-          <t>700156836</t>
+          <t>700158116</t>
         </is>
       </c>
     </row>
@@ -6131,7 +6131,7 @@
       </c>
       <c r="C335" s="2" t="inlineStr">
         <is>
-          <t>501136681</t>
+          <t>501137981</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6148,7 @@
       </c>
       <c r="C336" s="2" t="inlineStr">
         <is>
-          <t>700166081</t>
+          <t>700166080</t>
         </is>
       </c>
     </row>
@@ -6165,7 +6165,7 @@
       </c>
       <c r="C337" s="2" t="inlineStr">
         <is>
-          <t>501145086</t>
+          <t>501145085</t>
         </is>
       </c>
     </row>
@@ -6182,7 +6182,7 @@
       </c>
       <c r="C338" s="2" t="inlineStr">
         <is>
-          <t>700170081</t>
+          <t>700163414</t>
         </is>
       </c>
     </row>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="C339" s="2" t="inlineStr">
         <is>
-          <t>501149146</t>
+          <t>501143369</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6216,7 @@
       </c>
       <c r="C340" s="2" t="inlineStr">
         <is>
-          <t>700167282</t>
+          <t>700175794</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C341" s="2" t="inlineStr">
         <is>
-          <t>501146297</t>
+          <t>501154959</t>
         </is>
       </c>
     </row>
@@ -6250,7 +6250,7 @@
       </c>
       <c r="C342" s="2" t="inlineStr">
         <is>
-          <t>700178274</t>
+          <t>700166266</t>
         </is>
       </c>
     </row>
@@ -6267,7 +6267,7 @@
       </c>
       <c r="C343" s="2" t="inlineStr">
         <is>
-          <t>501157139</t>
+          <t>501145261</t>
         </is>
       </c>
     </row>
@@ -6284,7 +6284,7 @@
       </c>
       <c r="C344" s="2" t="inlineStr">
         <is>
-          <t>700168419</t>
+          <t>700174712</t>
         </is>
       </c>
     </row>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="C345" s="2" t="inlineStr">
         <is>
-          <t>501147464</t>
+          <t>501153857</t>
         </is>
       </c>
     </row>
@@ -6318,7 +6318,7 @@
       </c>
       <c r="C346" s="2" t="inlineStr">
         <is>
-          <t>700176290</t>
+          <t>700156749</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
       </c>
       <c r="C347" s="2" t="inlineStr">
         <is>
-          <t>501155485</t>
+          <t>501136584</t>
         </is>
       </c>
     </row>
@@ -6352,7 +6352,7 @@
       </c>
       <c r="C348" s="2" t="inlineStr">
         <is>
-          <t>700176933</t>
+          <t>700180527</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="C349" s="2" t="inlineStr">
         <is>
-          <t>501155828</t>
+          <t>501159412</t>
         </is>
       </c>
     </row>
@@ -6386,7 +6386,7 @@
       </c>
       <c r="C350" s="2" t="inlineStr">
         <is>
-          <t>700173236</t>
+          <t>700172573</t>
         </is>
       </c>
     </row>
@@ -6403,7 +6403,7 @@
       </c>
       <c r="C351" s="2" t="inlineStr">
         <is>
-          <t>501152361</t>
+          <t>501151688</t>
         </is>
       </c>
     </row>
@@ -6420,7 +6420,7 @@
       </c>
       <c r="C352" s="2" t="inlineStr">
         <is>
-          <t>700180074</t>
+          <t>700178224</t>
         </is>
       </c>
     </row>
@@ -6437,7 +6437,7 @@
       </c>
       <c r="C353" s="2" t="inlineStr">
         <is>
-          <t>501158939</t>
+          <t>501157089</t>
         </is>
       </c>
     </row>
@@ -6454,7 +6454,7 @@
       </c>
       <c r="C354" s="2" t="inlineStr">
         <is>
-          <t>700173850</t>
+          <t>700177069</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="C355" s="2" t="inlineStr">
         <is>
-          <t>501152975</t>
+          <t>501155967</t>
         </is>
       </c>
     </row>
@@ -6488,7 +6488,7 @@
       </c>
       <c r="C356" s="2" t="inlineStr">
         <is>
-          <t>700162387</t>
+          <t>700179574</t>
         </is>
       </c>
     </row>
@@ -6505,7 +6505,7 @@
       </c>
       <c r="C357" s="2" t="inlineStr">
         <is>
-          <t>501142092</t>
+          <t>501158449</t>
         </is>
       </c>
     </row>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="C358" s="2" t="inlineStr">
         <is>
-          <t>700168420</t>
+          <t>700161071</t>
         </is>
       </c>
     </row>
@@ -6539,7 +6539,7 @@
       </c>
       <c r="C359" s="2" t="inlineStr">
         <is>
-          <t>501147465</t>
+          <t>501140686</t>
         </is>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
       </c>
       <c r="C360" s="2" t="inlineStr">
         <is>
-          <t>700178224</t>
+          <t>700077050</t>
         </is>
       </c>
     </row>
@@ -6573,7 +6573,7 @@
       </c>
       <c r="C361" s="2" t="inlineStr">
         <is>
-          <t>501157089</t>
+          <t>501035584</t>
         </is>
       </c>
     </row>
@@ -6590,7 +6590,7 @@
       </c>
       <c r="C362" s="2" t="inlineStr">
         <is>
-          <t>700177002</t>
+          <t>700177730</t>
         </is>
       </c>
     </row>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="C363" s="2" t="inlineStr">
         <is>
-          <t>501155897</t>
+          <t>501156635</t>
         </is>
       </c>
     </row>
@@ -6624,7 +6624,7 @@
       </c>
       <c r="C364" s="2" t="inlineStr">
         <is>
-          <t>700175163</t>
+          <t>700177271</t>
         </is>
       </c>
     </row>
@@ -6641,7 +6641,7 @@
       </c>
       <c r="C365" s="2" t="inlineStr">
         <is>
-          <t>501154328</t>
+          <t>501156176</t>
         </is>
       </c>
     </row>
@@ -6658,7 +6658,7 @@
       </c>
       <c r="C366" s="2" t="inlineStr">
         <is>
-          <t>700177330</t>
+          <t>700173256</t>
         </is>
       </c>
     </row>
@@ -6675,7 +6675,7 @@
       </c>
       <c r="C367" s="2" t="inlineStr">
         <is>
-          <t>501156235</t>
+          <t>501152381</t>
         </is>
       </c>
     </row>
@@ -6692,7 +6692,7 @@
       </c>
       <c r="C368" s="2" t="inlineStr">
         <is>
-          <t>700161535</t>
+          <t>700176117</t>
         </is>
       </c>
     </row>
@@ -6709,7 +6709,7 @@
       </c>
       <c r="C369" s="2" t="inlineStr">
         <is>
-          <t>501141170</t>
+          <t>501155292</t>
         </is>
       </c>
     </row>
@@ -6726,7 +6726,7 @@
       </c>
       <c r="C370" s="2" t="inlineStr">
         <is>
-          <t>700177303</t>
+          <t>700157608</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6743,7 @@
       </c>
       <c r="C371" s="2" t="inlineStr">
         <is>
-          <t>501156208</t>
+          <t>501137443</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6760,7 @@
       </c>
       <c r="C372" s="2" t="inlineStr">
         <is>
-          <t>700175778</t>
+          <t>700178130</t>
         </is>
       </c>
     </row>
@@ -6777,7 +6777,7 @@
       </c>
       <c r="C373" s="2" t="inlineStr">
         <is>
-          <t>501154953</t>
+          <t>501156995</t>
         </is>
       </c>
     </row>
@@ -6794,7 +6794,7 @@
       </c>
       <c r="C374" s="2" t="inlineStr">
         <is>
-          <t>700167289</t>
+          <t>700177675</t>
         </is>
       </c>
     </row>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="C375" s="2" t="inlineStr">
         <is>
-          <t>501146304</t>
+          <t>501156580</t>
         </is>
       </c>
     </row>
@@ -6828,7 +6828,7 @@
       </c>
       <c r="C376" s="2" t="inlineStr">
         <is>
-          <t>700173543</t>
+          <t>700161073</t>
         </is>
       </c>
     </row>
@@ -6845,7 +6845,7 @@
       </c>
       <c r="C377" s="2" t="inlineStr">
         <is>
-          <t>501152668</t>
+          <t>501140688</t>
         </is>
       </c>
     </row>
@@ -6862,7 +6862,7 @@
       </c>
       <c r="C378" s="2" t="inlineStr">
         <is>
-          <t>700177270</t>
+          <t>700177903</t>
         </is>
       </c>
     </row>
@@ -6879,7 +6879,7 @@
       </c>
       <c r="C379" s="2" t="inlineStr">
         <is>
-          <t>501156175</t>
+          <t>501156808</t>
         </is>
       </c>
     </row>
@@ -6896,7 +6896,7 @@
       </c>
       <c r="C380" s="2" t="inlineStr">
         <is>
-          <t>700176117</t>
+          <t>700177306</t>
         </is>
       </c>
     </row>
@@ -6913,7 +6913,7 @@
       </c>
       <c r="C381" s="2" t="inlineStr">
         <is>
-          <t>501155292</t>
+          <t>501156211</t>
         </is>
       </c>
     </row>
@@ -6930,7 +6930,7 @@
       </c>
       <c r="C382" s="2" t="inlineStr">
         <is>
-          <t>700172038</t>
+          <t>700179263</t>
         </is>
       </c>
     </row>
@@ -6947,7 +6947,7 @@
       </c>
       <c r="C383" s="2" t="inlineStr">
         <is>
-          <t>501151143</t>
+          <t>501158128</t>
         </is>
       </c>
     </row>
@@ -6964,7 +6964,7 @@
       </c>
       <c r="C384" s="2" t="inlineStr">
         <is>
-          <t>700177743</t>
+          <t>700166081</t>
         </is>
       </c>
     </row>
@@ -6981,7 +6981,7 @@
       </c>
       <c r="C385" s="2" t="inlineStr">
         <is>
-          <t>501156648</t>
+          <t>501145086</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="C386" s="2" t="inlineStr">
         <is>
-          <t>700157609</t>
+          <t>700178505</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7015,7 @@
       </c>
       <c r="C387" s="2" t="inlineStr">
         <is>
-          <t>501137444</t>
+          <t>501157370</t>
         </is>
       </c>
     </row>
@@ -7032,7 +7032,7 @@
       </c>
       <c r="C388" s="2" t="inlineStr">
         <is>
-          <t>700177915</t>
+          <t>700173543</t>
         </is>
       </c>
     </row>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="C389" s="2" t="inlineStr">
         <is>
-          <t>501156820</t>
+          <t>501152668</t>
         </is>
       </c>
     </row>
@@ -7066,7 +7066,7 @@
       </c>
       <c r="C390" s="2" t="inlineStr">
         <is>
-          <t>700179573</t>
+          <t>700161535</t>
         </is>
       </c>
     </row>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C391" s="2" t="inlineStr">
         <is>
-          <t>501158448</t>
+          <t>501141170</t>
         </is>
       </c>
     </row>
@@ -7100,7 +7100,7 @@
       </c>
       <c r="C392" s="2" t="inlineStr">
         <is>
-          <t>700177310</t>
+          <t>700177680</t>
         </is>
       </c>
     </row>
@@ -7117,7 +7117,7 @@
       </c>
       <c r="C393" s="2" t="inlineStr">
         <is>
-          <t>501156215</t>
+          <t>501156585</t>
         </is>
       </c>
     </row>
@@ -7134,7 +7134,7 @@
       </c>
       <c r="C394" s="2" t="inlineStr">
         <is>
-          <t>700158791</t>
+          <t>700177310</t>
         </is>
       </c>
     </row>
@@ -7151,7 +7151,7 @@
       </c>
       <c r="C395" s="2" t="inlineStr">
         <is>
-          <t>501138635</t>
+          <t>501156215</t>
         </is>
       </c>
     </row>
@@ -7168,7 +7168,7 @@
       </c>
       <c r="C396" s="2" t="inlineStr">
         <is>
-          <t>700158787</t>
+          <t>700178232</t>
         </is>
       </c>
     </row>
@@ -7185,7 +7185,7 @@
       </c>
       <c r="C397" s="2" t="inlineStr">
         <is>
-          <t>501138631</t>
+          <t>501157097</t>
         </is>
       </c>
     </row>
@@ -7202,7 +7202,7 @@
       </c>
       <c r="C398" s="2" t="inlineStr">
         <is>
-          <t>700158788</t>
+          <t>700179114</t>
         </is>
       </c>
     </row>
@@ -7219,7 +7219,7 @@
       </c>
       <c r="C399" s="2" t="inlineStr">
         <is>
-          <t>501138632</t>
+          <t>501157979</t>
         </is>
       </c>
     </row>
@@ -7236,7 +7236,7 @@
       </c>
       <c r="C400" s="2" t="inlineStr">
         <is>
-          <t>700177070</t>
+          <t>700161494</t>
         </is>
       </c>
     </row>
@@ -7253,7 +7253,7 @@
       </c>
       <c r="C401" s="2" t="inlineStr">
         <is>
-          <t>501155988</t>
+          <t>501141109</t>
         </is>
       </c>
     </row>
@@ -7270,7 +7270,7 @@
       </c>
       <c r="C402" s="2" t="inlineStr">
         <is>
-          <t>700172271</t>
+          <t>700177311</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="C403" s="2" t="inlineStr">
         <is>
-          <t>501151376</t>
+          <t>501156216</t>
         </is>
       </c>
     </row>
@@ -7304,7 +7304,7 @@
       </c>
       <c r="C404" s="2" t="inlineStr">
         <is>
-          <t>700165632</t>
+          <t>700158788</t>
         </is>
       </c>
     </row>
@@ -7321,7 +7321,7 @@
       </c>
       <c r="C405" s="2" t="inlineStr">
         <is>
-          <t>501144627</t>
+          <t>501138632</t>
         </is>
       </c>
     </row>
@@ -7338,7 +7338,7 @@
       </c>
       <c r="C406" s="2" t="inlineStr">
         <is>
-          <t>700173940</t>
+          <t>700177107</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7355,7 @@
       </c>
       <c r="C407" s="2" t="inlineStr">
         <is>
-          <t>501153075</t>
+          <t>501156012</t>
         </is>
       </c>
     </row>
@@ -7372,7 +7372,7 @@
       </c>
       <c r="C408" s="2" t="inlineStr">
         <is>
-          <t>700158116</t>
+          <t>700157609</t>
         </is>
       </c>
     </row>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="C409" s="2" t="inlineStr">
         <is>
-          <t>501137981</t>
+          <t>501137444</t>
         </is>
       </c>
     </row>
@@ -7406,7 +7406,7 @@
       </c>
       <c r="C410" s="2" t="inlineStr">
         <is>
-          <t>700161462</t>
+          <t>700162386</t>
         </is>
       </c>
     </row>
@@ -7423,7 +7423,7 @@
       </c>
       <c r="C411" s="2" t="inlineStr">
         <is>
-          <t>501141077</t>
+          <t>501142091</t>
         </is>
       </c>
     </row>
@@ -7440,7 +7440,7 @@
       </c>
       <c r="C412" s="2" t="inlineStr">
         <is>
-          <t>700179112</t>
+          <t>700177917</t>
         </is>
       </c>
     </row>
@@ -7457,7 +7457,7 @@
       </c>
       <c r="C413" s="2" t="inlineStr">
         <is>
-          <t>501157977</t>
+          <t>501156822</t>
         </is>
       </c>
     </row>
@@ -7474,7 +7474,7 @@
       </c>
       <c r="C414" s="2" t="inlineStr">
         <is>
-          <t>700176012</t>
+          <t>700177005</t>
         </is>
       </c>
     </row>
@@ -7491,7 +7491,7 @@
       </c>
       <c r="C415" s="2" t="inlineStr">
         <is>
-          <t>501155187</t>
+          <t>501155900</t>
         </is>
       </c>
     </row>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="C416" s="2" t="inlineStr">
         <is>
-          <t>700178504</t>
+          <t>700177902</t>
         </is>
       </c>
     </row>
@@ -7525,7 +7525,7 @@
       </c>
       <c r="C417" s="2" t="inlineStr">
         <is>
-          <t>501157369</t>
+          <t>501156807</t>
         </is>
       </c>
     </row>
@@ -7542,7 +7542,7 @@
       </c>
       <c r="C418" s="2" t="inlineStr">
         <is>
-          <t>700172573</t>
+          <t>700175163</t>
         </is>
       </c>
     </row>
@@ -7559,7 +7559,7 @@
       </c>
       <c r="C419" s="2" t="inlineStr">
         <is>
-          <t>501151688</t>
+          <t>501154328</t>
         </is>
       </c>
     </row>
@@ -7576,7 +7576,7 @@
       </c>
       <c r="C420" s="2" t="inlineStr">
         <is>
-          <t>700178789</t>
+          <t>700179116</t>
         </is>
       </c>
     </row>
@@ -7593,7 +7593,7 @@
       </c>
       <c r="C421" s="2" t="inlineStr">
         <is>
-          <t>501157664</t>
+          <t>501157981</t>
         </is>
       </c>
     </row>
@@ -7610,7 +7610,7 @@
       </c>
       <c r="C422" s="2" t="inlineStr">
         <is>
-          <t>700159804</t>
+          <t>700156748</t>
         </is>
       </c>
     </row>
@@ -7627,7 +7627,7 @@
       </c>
       <c r="C423" s="2" t="inlineStr">
         <is>
-          <t>501139679</t>
+          <t>501136583</t>
         </is>
       </c>
     </row>
@@ -7644,7 +7644,7 @@
       </c>
       <c r="C424" s="2" t="inlineStr">
         <is>
-          <t>700157673</t>
+          <t>700176046</t>
         </is>
       </c>
     </row>
@@ -7661,7 +7661,7 @@
       </c>
       <c r="C425" s="2" t="inlineStr">
         <is>
-          <t>501137508</t>
+          <t>501155221</t>
         </is>
       </c>
     </row>
@@ -7678,7 +7678,7 @@
       </c>
       <c r="C426" s="2" t="inlineStr">
         <is>
-          <t>700165912</t>
+          <t>700177465</t>
         </is>
       </c>
     </row>
@@ -7695,7 +7695,7 @@
       </c>
       <c r="C427" s="2" t="inlineStr">
         <is>
-          <t>501144917</t>
+          <t>501156370</t>
         </is>
       </c>
     </row>
@@ -7712,7 +7712,7 @@
       </c>
       <c r="C428" s="2" t="inlineStr">
         <is>
-          <t>700175776</t>
+          <t>700162385</t>
         </is>
       </c>
     </row>
@@ -7729,7 +7729,7 @@
       </c>
       <c r="C429" s="2" t="inlineStr">
         <is>
-          <t>501154951</t>
+          <t>501142090</t>
         </is>
       </c>
     </row>
@@ -7746,7 +7746,7 @@
       </c>
       <c r="C430" s="2" t="inlineStr">
         <is>
-          <t>700177917</t>
+          <t>700165715</t>
         </is>
       </c>
     </row>
@@ -7763,7 +7763,7 @@
       </c>
       <c r="C431" s="2" t="inlineStr">
         <is>
-          <t>501156822</t>
+          <t>501144720</t>
         </is>
       </c>
     </row>
@@ -7780,7 +7780,7 @@
       </c>
       <c r="C432" s="2" t="inlineStr">
         <is>
-          <t>700156837</t>
+          <t>700162041</t>
         </is>
       </c>
     </row>
@@ -7797,7 +7797,7 @@
       </c>
       <c r="C433" s="2" t="inlineStr">
         <is>
-          <t>501136682</t>
+          <t>501141716</t>
         </is>
       </c>
     </row>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="C434" s="2" t="inlineStr">
         <is>
-          <t>700169344</t>
+          <t>700178492</t>
         </is>
       </c>
     </row>
@@ -7831,7 +7831,7 @@
       </c>
       <c r="C435" s="2" t="inlineStr">
         <is>
-          <t>501148399</t>
+          <t>501157357</t>
         </is>
       </c>
     </row>
@@ -7848,7 +7848,7 @@
       </c>
       <c r="C436" s="2" t="inlineStr">
         <is>
-          <t>700174411</t>
+          <t>700175725</t>
         </is>
       </c>
     </row>
@@ -7865,7 +7865,7 @@
       </c>
       <c r="C437" s="2" t="inlineStr">
         <is>
-          <t>501153556</t>
+          <t>501154900</t>
         </is>
       </c>
     </row>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="C438" s="2" t="inlineStr">
         <is>
-          <t>700177465</t>
+          <t>700177743</t>
         </is>
       </c>
     </row>
@@ -7899,7 +7899,7 @@
       </c>
       <c r="C439" s="2" t="inlineStr">
         <is>
-          <t>501156370</t>
+          <t>501156648</t>
         </is>
       </c>
     </row>
@@ -7916,7 +7916,7 @@
       </c>
       <c r="C440" s="2" t="inlineStr">
         <is>
-          <t>700177677</t>
+          <t>700176947</t>
         </is>
       </c>
     </row>
@@ -7933,7 +7933,7 @@
       </c>
       <c r="C441" s="2" t="inlineStr">
         <is>
-          <t>501156583</t>
+          <t>501155842</t>
         </is>
       </c>
     </row>
@@ -7950,7 +7950,7 @@
       </c>
       <c r="C442" s="2" t="inlineStr">
         <is>
-          <t>700077050</t>
+          <t>700165912</t>
         </is>
       </c>
     </row>
@@ -7967,7 +7967,7 @@
       </c>
       <c r="C443" s="2" t="inlineStr">
         <is>
-          <t>501035584</t>
+          <t>501144917</t>
         </is>
       </c>
     </row>
@@ -7984,7 +7984,7 @@
       </c>
       <c r="C444" s="2" t="inlineStr">
         <is>
-          <t>700165629</t>
+          <t>700159805</t>
         </is>
       </c>
     </row>
@@ -8001,7 +8001,7 @@
       </c>
       <c r="C445" s="2" t="inlineStr">
         <is>
-          <t>501144624</t>
+          <t>501139680</t>
         </is>
       </c>
     </row>
@@ -8018,7 +8018,7 @@
       </c>
       <c r="C446" s="2" t="inlineStr">
         <is>
-          <t>700177896</t>
+          <t>700180073</t>
         </is>
       </c>
     </row>
@@ -8035,7 +8035,7 @@
       </c>
       <c r="C447" s="2" t="inlineStr">
         <is>
-          <t>501156801</t>
+          <t>501158938</t>
         </is>
       </c>
     </row>
@@ -8052,7 +8052,7 @@
       </c>
       <c r="C448" s="2" t="inlineStr">
         <is>
-          <t>700177321</t>
+          <t>700176148</t>
         </is>
       </c>
     </row>
@@ -8069,7 +8069,7 @@
       </c>
       <c r="C449" s="2" t="inlineStr">
         <is>
-          <t>501156226</t>
+          <t>501155323</t>
         </is>
       </c>
     </row>
@@ -8086,7 +8086,7 @@
       </c>
       <c r="C450" s="2" t="inlineStr">
         <is>
-          <t>700176145</t>
+          <t>700176144</t>
         </is>
       </c>
     </row>
@@ -8103,7 +8103,7 @@
       </c>
       <c r="C451" s="2" t="inlineStr">
         <is>
-          <t>501155320</t>
+          <t>501155319</t>
         </is>
       </c>
     </row>
@@ -8120,7 +8120,7 @@
       </c>
       <c r="C452" s="2" t="inlineStr">
         <is>
-          <t>700161072</t>
+          <t>700177360</t>
         </is>
       </c>
     </row>
@@ -8137,7 +8137,7 @@
       </c>
       <c r="C453" s="2" t="inlineStr">
         <is>
-          <t>501140687</t>
+          <t>501156265</t>
         </is>
       </c>
     </row>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="C454" s="2" t="inlineStr">
         <is>
-          <t>700180032</t>
+          <t>700178231</t>
         </is>
       </c>
     </row>
@@ -8171,7 +8171,7 @@
       </c>
       <c r="C455" s="2" t="inlineStr">
         <is>
-          <t>501158907</t>
+          <t>501157096</t>
         </is>
       </c>
     </row>
@@ -8188,7 +8188,7 @@
       </c>
       <c r="C456" s="2" t="inlineStr">
         <is>
-          <t>700176144</t>
+          <t>700176118</t>
         </is>
       </c>
     </row>
@@ -8205,7 +8205,7 @@
       </c>
       <c r="C457" s="2" t="inlineStr">
         <is>
-          <t>501155319</t>
+          <t>501155293</t>
         </is>
       </c>
     </row>
@@ -8222,7 +8222,7 @@
       </c>
       <c r="C458" s="2" t="inlineStr">
         <is>
-          <t>700178231</t>
+          <t>700177330</t>
         </is>
       </c>
     </row>
@@ -8239,7 +8239,7 @@
       </c>
       <c r="C459" s="2" t="inlineStr">
         <is>
-          <t>501157096</t>
+          <t>501156235</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8256,7 @@
       </c>
       <c r="C460" s="2" t="inlineStr">
         <is>
-          <t>700174493</t>
+          <t>700162387</t>
         </is>
       </c>
     </row>
@@ -8273,7 +8273,7 @@
       </c>
       <c r="C461" s="2" t="inlineStr">
         <is>
-          <t>501153638</t>
+          <t>501142092</t>
         </is>
       </c>
     </row>
@@ -8290,7 +8290,7 @@
       </c>
       <c r="C462" s="2" t="inlineStr">
         <is>
-          <t>700177730</t>
+          <t>700177639</t>
         </is>
       </c>
     </row>
@@ -8307,7 +8307,7 @@
       </c>
       <c r="C463" s="2" t="inlineStr">
         <is>
-          <t>501156635</t>
+          <t>501156544</t>
         </is>
       </c>
     </row>
@@ -8324,7 +8324,7 @@
       </c>
       <c r="C464" s="2" t="inlineStr">
         <is>
-          <t>700179545</t>
+          <t>700174410</t>
         </is>
       </c>
     </row>
@@ -8341,7 +8341,7 @@
       </c>
       <c r="C465" s="2" t="inlineStr">
         <is>
-          <t>501158420</t>
+          <t>501153555</t>
         </is>
       </c>
     </row>
@@ -8358,7 +8358,7 @@
       </c>
       <c r="C466" s="2" t="inlineStr">
         <is>
-          <t>700176047</t>
+          <t>700161462</t>
         </is>
       </c>
     </row>
@@ -8375,7 +8375,7 @@
       </c>
       <c r="C467" s="2" t="inlineStr">
         <is>
-          <t>501155222</t>
+          <t>501141077</t>
         </is>
       </c>
     </row>
@@ -8392,7 +8392,7 @@
       </c>
       <c r="C468" s="2" t="inlineStr">
         <is>
-          <t>700179621</t>
+          <t>700178600</t>
         </is>
       </c>
     </row>
@@ -8409,7 +8409,7 @@
       </c>
       <c r="C469" s="2" t="inlineStr">
         <is>
-          <t>501158496</t>
+          <t>501157467</t>
         </is>
       </c>
     </row>
@@ -8426,7 +8426,7 @@
       </c>
       <c r="C470" s="2" t="inlineStr">
         <is>
-          <t>700172267</t>
+          <t>700172271</t>
         </is>
       </c>
     </row>
@@ -8443,7 +8443,7 @@
       </c>
       <c r="C471" s="2" t="inlineStr">
         <is>
-          <t>501151372</t>
+          <t>501151376</t>
         </is>
       </c>
     </row>
@@ -8460,7 +8460,7 @@
       </c>
       <c r="C472" s="2" t="inlineStr">
         <is>
-          <t>700160396</t>
+          <t>700169347</t>
         </is>
       </c>
     </row>
@@ -8477,7 +8477,7 @@
       </c>
       <c r="C473" s="2" t="inlineStr">
         <is>
-          <t>501139971</t>
+          <t>501148402</t>
         </is>
       </c>
     </row>
@@ -8494,7 +8494,7 @@
       </c>
       <c r="C474" s="2" t="inlineStr">
         <is>
-          <t>700174572</t>
+          <t>700180033</t>
         </is>
       </c>
     </row>
@@ -8511,7 +8511,7 @@
       </c>
       <c r="C475" s="2" t="inlineStr">
         <is>
-          <t>501153727</t>
+          <t>501158908</t>
         </is>
       </c>
     </row>
@@ -8528,7 +8528,7 @@
       </c>
       <c r="C476" s="2" t="inlineStr">
         <is>
-          <t>700177106</t>
+          <t>700161534</t>
         </is>
       </c>
     </row>
@@ -8545,7 +8545,7 @@
       </c>
       <c r="C477" s="2" t="inlineStr">
         <is>
-          <t>501156011</t>
+          <t>501141169</t>
         </is>
       </c>
     </row>
@@ -8562,7 +8562,7 @@
       </c>
       <c r="C478" s="2" t="inlineStr">
         <is>
-          <t>700178232</t>
+          <t>700157674</t>
         </is>
       </c>
     </row>
@@ -8579,7 +8579,7 @@
       </c>
       <c r="C479" s="2" t="inlineStr">
         <is>
-          <t>501157097</t>
+          <t>501137509</t>
         </is>
       </c>
     </row>
@@ -8596,7 +8596,7 @@
       </c>
       <c r="C480" s="2" t="inlineStr">
         <is>
-          <t>700177727</t>
+          <t>700158115</t>
         </is>
       </c>
     </row>
@@ -8613,7 +8613,7 @@
       </c>
       <c r="C481" s="2" t="inlineStr">
         <is>
-          <t>501156632</t>
+          <t>501137980</t>
         </is>
       </c>
     </row>
@@ -8630,7 +8630,7 @@
       </c>
       <c r="C482" s="2" t="inlineStr">
         <is>
-          <t>700177675</t>
+          <t>700180042</t>
         </is>
       </c>
     </row>
@@ -8647,7 +8647,7 @@
       </c>
       <c r="C483" s="2" t="inlineStr">
         <is>
-          <t>501156580</t>
+          <t>501158917</t>
         </is>
       </c>
     </row>
@@ -8664,7 +8664,7 @@
       </c>
       <c r="C484" s="2" t="inlineStr">
         <is>
-          <t>700179113</t>
+          <t>700165632</t>
         </is>
       </c>
     </row>
@@ -8681,7 +8681,7 @@
       </c>
       <c r="C485" s="2" t="inlineStr">
         <is>
-          <t>501157978</t>
+          <t>501144627</t>
         </is>
       </c>
     </row>
@@ -8698,7 +8698,7 @@
       </c>
       <c r="C486" s="2" t="inlineStr">
         <is>
-          <t>700161534</t>
+          <t>700175781</t>
         </is>
       </c>
     </row>
@@ -8715,7 +8715,7 @@
       </c>
       <c r="C487" s="2" t="inlineStr">
         <is>
-          <t>501141169</t>
+          <t>501154956</t>
         </is>
       </c>
     </row>
@@ -8732,7 +8732,7 @@
       </c>
       <c r="C488" s="2" t="inlineStr">
         <is>
-          <t>700180041</t>
+          <t>700179533</t>
         </is>
       </c>
     </row>
@@ -8749,7 +8749,7 @@
       </c>
       <c r="C489" s="2" t="inlineStr">
         <is>
-          <t>501158916</t>
+          <t>501158408</t>
         </is>
       </c>
     </row>
@@ -8766,7 +8766,7 @@
       </c>
       <c r="C490" s="2" t="inlineStr">
         <is>
-          <t>700156748</t>
+          <t>700177896</t>
         </is>
       </c>
     </row>
@@ -8783,7 +8783,7 @@
       </c>
       <c r="C491" s="2" t="inlineStr">
         <is>
-          <t>501136583</t>
+          <t>501156801</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="C492" s="2" t="inlineStr">
         <is>
-          <t>700172574</t>
+          <t>700177726</t>
         </is>
       </c>
     </row>
@@ -8817,7 +8817,7 @@
       </c>
       <c r="C493" s="2" t="inlineStr">
         <is>
-          <t>501151689</t>
+          <t>501156631</t>
         </is>
       </c>
     </row>
@@ -8834,7 +8834,7 @@
       </c>
       <c r="C494" s="2" t="inlineStr">
         <is>
-          <t>700172270</t>
+          <t>700173236</t>
         </is>
       </c>
     </row>
@@ -8851,7 +8851,7 @@
       </c>
       <c r="C495" s="2" t="inlineStr">
         <is>
-          <t>501151375</t>
+          <t>501152361</t>
         </is>
       </c>
     </row>
@@ -8868,7 +8868,7 @@
       </c>
       <c r="C496" s="2" t="inlineStr">
         <is>
-          <t>700179263</t>
+          <t>700175761</t>
         </is>
       </c>
     </row>
@@ -8885,7 +8885,7 @@
       </c>
       <c r="C497" s="2" t="inlineStr">
         <is>
-          <t>501158128</t>
+          <t>501154936</t>
         </is>
       </c>
     </row>
@@ -8902,7 +8902,7 @@
       </c>
       <c r="C498" s="2" t="inlineStr">
         <is>
-          <t>700173797</t>
+          <t>700177106</t>
         </is>
       </c>
     </row>
@@ -8919,7 +8919,7 @@
       </c>
       <c r="C499" s="2" t="inlineStr">
         <is>
-          <t>501152922</t>
+          <t>501156011</t>
         </is>
       </c>
     </row>
@@ -8936,7 +8936,7 @@
       </c>
       <c r="C500" s="2" t="inlineStr">
         <is>
-          <t>700173796</t>
+          <t>700179621</t>
         </is>
       </c>
     </row>
@@ -8953,7 +8953,7 @@
       </c>
       <c r="C501" s="2" t="inlineStr">
         <is>
-          <t>501152921</t>
+          <t>501158496</t>
         </is>
       </c>
     </row>
@@ -8970,7 +8970,7 @@
       </c>
       <c r="C502" s="2" t="inlineStr">
         <is>
-          <t>700173256</t>
+          <t>700161493</t>
         </is>
       </c>
     </row>
@@ -8987,7 +8987,7 @@
       </c>
       <c r="C503" s="2" t="inlineStr">
         <is>
-          <t>501152381</t>
+          <t>501141108</t>
         </is>
       </c>
     </row>
@@ -9004,7 +9004,7 @@
       </c>
       <c r="C504" s="2" t="inlineStr">
         <is>
-          <t>700177360</t>
+          <t>700178230</t>
         </is>
       </c>
     </row>
@@ -9021,7 +9021,7 @@
       </c>
       <c r="C505" s="2" t="inlineStr">
         <is>
-          <t>501156265</t>
+          <t>501157095</t>
         </is>
       </c>
     </row>
@@ -9038,7 +9038,7 @@
       </c>
       <c r="C506" s="2" t="inlineStr">
         <is>
-          <t>700177986</t>
+          <t>700177895</t>
         </is>
       </c>
     </row>
@@ -9055,7 +9055,7 @@
       </c>
       <c r="C507" s="2" t="inlineStr">
         <is>
-          <t>501156841</t>
+          <t>501156800</t>
         </is>
       </c>
     </row>
@@ -9072,7 +9072,7 @@
       </c>
       <c r="C508" s="2" t="inlineStr">
         <is>
-          <t>700174410</t>
+          <t>700178131</t>
         </is>
       </c>
     </row>
@@ -9089,7 +9089,7 @@
       </c>
       <c r="C509" s="2" t="inlineStr">
         <is>
-          <t>501153555</t>
+          <t>501156996</t>
         </is>
       </c>
     </row>

</xml_diff>